<commit_message>
Incorporar revision de previsiones Q4 de Irene a matrices presupuestarias, informe de cambios y dashboard
</commit_message>
<xml_diff>
--- a/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_CONSOLIDADO.xlsx
+++ b/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_CONSOLIDADO.xlsx
@@ -12988,12 +12988,16 @@
         <f>IF(F10&gt;0, G10/F10, IF(G10&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J10" s="33" t="inlineStr"/>
+      <c r="J10" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K10" s="34" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="35" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M10" s="34" t="n">
         <v>0</v>
@@ -13005,7 +13009,7 @@
         <v>200</v>
       </c>
       <c r="P10" s="35" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="Q10" s="12">
         <f>K10+M10+O10</f>
@@ -13019,7 +13023,7 @@
         <f>R10-Q10</f>
         <v/>
       </c>
-      <c r="T10" s="37" t="inlineStr"/>
+      <c r="T10" s="37" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="11" t="inlineStr">
@@ -13091,7 +13095,7 @@
         <f>R11-Q11</f>
         <v/>
       </c>
-      <c r="T11" s="37" t="inlineStr"/>
+      <c r="T11" s="37" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="11" t="inlineStr">
@@ -13128,24 +13132,28 @@
         <f>IF(F12&gt;0, G12/F12, IF(G12&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J12" s="33" t="inlineStr"/>
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K12" s="34" t="n">
         <v>5060</v>
       </c>
       <c r="L12" s="35" t="n">
-        <v>5060</v>
+        <v>3840</v>
       </c>
       <c r="M12" s="34" t="n">
         <v>1920</v>
       </c>
       <c r="N12" s="35" t="n">
-        <v>1920</v>
+        <v>3200</v>
       </c>
       <c r="O12" s="34" t="n">
         <v>3200</v>
       </c>
       <c r="P12" s="35" t="n">
-        <v>3200</v>
+        <v>3840</v>
       </c>
       <c r="Q12" s="12">
         <f>K12+M12+O12</f>
@@ -13159,7 +13167,11 @@
         <f>R12-Q12</f>
         <v/>
       </c>
-      <c r="T12" s="37" t="inlineStr"/>
+      <c r="T12" s="37" t="inlineStr">
+        <is>
+          <t>Han ido adelantados en compras, tienen en stock más de 6000 l y las plantaciones van este año más atrasadas.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="11" t="inlineStr">
@@ -13196,12 +13208,16 @@
         <f>IF(F13&gt;0, G13/F13, IF(G13&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J13" s="33" t="inlineStr"/>
+      <c r="J13" s="33" t="inlineStr">
+        <is>
+          <t>Mayor venta en envases 20l</t>
+        </is>
+      </c>
       <c r="K13" s="34" t="n">
         <v>300</v>
       </c>
       <c r="L13" s="35" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="M13" s="34" t="n">
         <v>0</v>
@@ -13227,7 +13243,11 @@
         <f>R13-Q13</f>
         <v/>
       </c>
-      <c r="T13" s="37" t="inlineStr"/>
+      <c r="T13" s="37" t="inlineStr">
+        <is>
+          <t>Esta saliendo m´sa en formato 20 l</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="11" t="inlineStr">
@@ -13264,18 +13284,22 @@
         <f>IF(F14&gt;0, G14/F14, IF(G14&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J14" s="33" t="inlineStr"/>
+      <c r="J14" s="33" t="inlineStr">
+        <is>
+          <t>Adelanto de pedidos</t>
+        </is>
+      </c>
       <c r="K14" s="34" t="n">
         <v>640</v>
       </c>
       <c r="L14" s="35" t="n">
-        <v>640</v>
+        <v>1280</v>
       </c>
       <c r="M14" s="34" t="n">
         <v>960</v>
       </c>
       <c r="N14" s="35" t="n">
-        <v>960</v>
+        <v>640</v>
       </c>
       <c r="O14" s="34" t="n">
         <v>1280</v>
@@ -13295,7 +13319,7 @@
         <f>R14-Q14</f>
         <v/>
       </c>
-      <c r="T14" s="37" t="inlineStr"/>
+      <c r="T14" s="37" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
@@ -13332,7 +13356,7 @@
         <f>IF(F15&gt;0, G15/F15, IF(G15&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J15" s="33" t="inlineStr"/>
+      <c r="J15" s="33" t="n"/>
       <c r="K15" s="34" t="n">
         <v>0</v>
       </c>
@@ -13363,7 +13387,7 @@
         <f>R15-Q15</f>
         <v/>
       </c>
-      <c r="T15" s="37" t="inlineStr"/>
+      <c r="T15" s="37" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="11" t="inlineStr">
@@ -13400,7 +13424,7 @@
         <f>IF(F16&gt;0, G16/F16, IF(G16&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J16" s="33" t="inlineStr"/>
+      <c r="J16" s="33" t="n"/>
       <c r="K16" s="34" t="n">
         <v>100</v>
       </c>
@@ -13431,7 +13455,7 @@
         <f>R16-Q16</f>
         <v/>
       </c>
-      <c r="T16" s="37" t="inlineStr"/>
+      <c r="T16" s="37" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
@@ -13468,7 +13492,11 @@
         <f>IF(F17&gt;0, G17/F17, IF(G17&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J17" s="33" t="inlineStr"/>
+      <c r="J17" s="33" t="inlineStr">
+        <is>
+          <t>Campaña habitual</t>
+        </is>
+      </c>
       <c r="K17" s="34" t="n">
         <v>640</v>
       </c>
@@ -13499,7 +13527,7 @@
         <f>R17-Q17</f>
         <v/>
       </c>
-      <c r="T17" s="37" t="inlineStr"/>
+      <c r="T17" s="37" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="11" t="inlineStr">
@@ -13536,7 +13564,7 @@
         <f>IF(F18&gt;0, G18/F18, IF(G18&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J18" s="33" t="inlineStr"/>
+      <c r="J18" s="33" t="n"/>
       <c r="K18" s="34" t="n">
         <v>200</v>
       </c>
@@ -13567,7 +13595,7 @@
         <f>R18-Q18</f>
         <v/>
       </c>
-      <c r="T18" s="37" t="inlineStr"/>
+      <c r="T18" s="37" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="11" t="inlineStr">
@@ -13604,7 +13632,7 @@
         <f>IF(F19&gt;0, G19/F19, IF(G19&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J19" s="33" t="inlineStr"/>
+      <c r="J19" s="33" t="n"/>
       <c r="K19" s="34" t="n">
         <v>0</v>
       </c>
@@ -13635,7 +13663,11 @@
         <f>R19-Q19</f>
         <v/>
       </c>
-      <c r="T19" s="37" t="inlineStr"/>
+      <c r="T19" s="37" t="inlineStr">
+        <is>
+          <t>El stock es grande y la aplicación de este producto es bien avanzado el Q4</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="11" t="inlineStr">
@@ -13672,7 +13704,11 @@
         <f>IF(F20&gt;0, G20/F20, IF(G20&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J20" s="33" t="inlineStr"/>
+      <c r="J20" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K20" s="34" t="n">
         <v>120</v>
       </c>
@@ -13703,7 +13739,7 @@
         <f>R20-Q20</f>
         <v/>
       </c>
-      <c r="T20" s="37" t="inlineStr"/>
+      <c r="T20" s="37" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="11" t="inlineStr">
@@ -13740,7 +13776,11 @@
         <f>IF(F21&gt;0, G21/F21, IF(G21&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J21" s="33" t="inlineStr"/>
+      <c r="J21" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K21" s="34" t="n">
         <v>0</v>
       </c>
@@ -13751,13 +13791,13 @@
         <v>400</v>
       </c>
       <c r="N21" s="35" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="O21" s="34" t="n">
         <v>300</v>
       </c>
       <c r="P21" s="35" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="12">
         <f>K21+M21+O21</f>
@@ -13771,7 +13811,11 @@
         <f>R21-Q21</f>
         <v/>
       </c>
-      <c r="T21" s="37" t="inlineStr"/>
+      <c r="T21" s="37" t="inlineStr">
+        <is>
+          <t>Según cliente tienen bastante stcok.Van adelantados en compras (el pedido que se cuatriplicó).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="11" t="inlineStr">
@@ -13808,7 +13852,11 @@
         <f>IF(F22&gt;0, G22/F22, IF(G22&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J22" s="33" t="inlineStr"/>
+      <c r="J22" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K22" s="34" t="n">
         <v>0</v>
       </c>
@@ -13839,7 +13887,7 @@
         <f>R22-Q22</f>
         <v/>
       </c>
-      <c r="T22" s="37" t="inlineStr"/>
+      <c r="T22" s="37" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="11" t="inlineStr">
@@ -13876,24 +13924,28 @@
         <f>IF(F23&gt;0, G23/F23, IF(G23&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J23" s="33" t="inlineStr"/>
+      <c r="J23" s="33" t="inlineStr">
+        <is>
+          <t>Adelanto de pedidos</t>
+        </is>
+      </c>
       <c r="K23" s="34" t="n">
         <v>120</v>
       </c>
       <c r="L23" s="35" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="M23" s="34" t="n">
         <v>200</v>
       </c>
       <c r="N23" s="35" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="O23" s="34" t="n">
         <v>300</v>
       </c>
       <c r="P23" s="35" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="Q23" s="12">
         <f>K23+M23+O23</f>
@@ -13907,7 +13959,11 @@
         <f>R23-Q23</f>
         <v/>
       </c>
-      <c r="T23" s="37" t="inlineStr"/>
+      <c r="T23" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adelanto de pedidos, </t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="11" t="inlineStr">
@@ -13944,24 +14000,28 @@
         <f>IF(F24&gt;0, G24/F24, IF(G24&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J24" s="33" t="inlineStr"/>
+      <c r="J24" s="33" t="inlineStr">
+        <is>
+          <t>Adelanto de pedidos</t>
+        </is>
+      </c>
       <c r="K24" s="34" t="n">
         <v>850</v>
       </c>
       <c r="L24" s="35" t="n">
-        <v>850</v>
+        <v>750</v>
       </c>
       <c r="M24" s="34" t="n">
         <v>500</v>
       </c>
       <c r="N24" s="35" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="O24" s="34" t="n">
         <v>1200</v>
       </c>
       <c r="P24" s="35" t="n">
-        <v>1200</v>
+        <v>750</v>
       </c>
       <c r="Q24" s="12">
         <f>K24+M24+O24</f>
@@ -13975,7 +14035,11 @@
         <f>R24-Q24</f>
         <v/>
       </c>
-      <c r="T24" s="37" t="inlineStr"/>
+      <c r="T24" s="37" t="inlineStr">
+        <is>
+          <t>Van adelantado en pedidos</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="11" t="inlineStr">
@@ -14012,12 +14076,16 @@
         <f>IF(F25&gt;0, G25/F25, IF(G25&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J25" s="33" t="inlineStr"/>
+      <c r="J25" s="33" t="inlineStr">
+        <is>
+          <t>Adelanto de pedidos</t>
+        </is>
+      </c>
       <c r="K25" s="34" t="n">
         <v>4480</v>
       </c>
       <c r="L25" s="35" t="n">
-        <v>4480</v>
+        <v>3200</v>
       </c>
       <c r="M25" s="34" t="n">
         <v>2560</v>
@@ -14043,7 +14111,11 @@
         <f>R25-Q25</f>
         <v/>
       </c>
-      <c r="T25" s="37" t="inlineStr"/>
+      <c r="T25" s="37" t="inlineStr">
+        <is>
+          <t>Van adelantados en los pedidos</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="11" t="inlineStr">
@@ -14080,7 +14152,7 @@
         <f>IF(F26&gt;0, G26/F26, IF(G26&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J26" s="33" t="inlineStr"/>
+      <c r="J26" s="33" t="n"/>
       <c r="K26" s="34" t="n">
         <v>0</v>
       </c>
@@ -14111,7 +14183,7 @@
         <f>R26-Q26</f>
         <v/>
       </c>
-      <c r="T26" s="37" t="inlineStr"/>
+      <c r="T26" s="37" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="B27" s="11" t="inlineStr">
@@ -14148,7 +14220,7 @@
         <f>IF(F27&gt;0, G27/F27, IF(G27&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J27" s="33" t="inlineStr"/>
+      <c r="J27" s="33" t="n"/>
       <c r="K27" s="34" t="n">
         <v>0</v>
       </c>
@@ -14179,7 +14251,7 @@
         <f>R27-Q27</f>
         <v/>
       </c>
-      <c r="T27" s="37" t="inlineStr"/>
+      <c r="T27" s="37" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="B28" s="11" t="inlineStr">
@@ -14251,7 +14323,7 @@
         <f>R28-Q28</f>
         <v/>
       </c>
-      <c r="T28" s="37" t="inlineStr"/>
+      <c r="T28" s="37" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="11" t="inlineStr">
@@ -14288,7 +14360,11 @@
         <f>IF(F29&gt;0, G29/F29, IF(G29&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J29" s="33" t="inlineStr"/>
+      <c r="J29" s="33" t="inlineStr">
+        <is>
+          <t>Otro motivo</t>
+        </is>
+      </c>
       <c r="K29" s="34" t="n">
         <v>0</v>
       </c>
@@ -14319,7 +14395,7 @@
         <f>R29-Q29</f>
         <v/>
       </c>
-      <c r="T29" s="37" t="inlineStr"/>
+      <c r="T29" s="37" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="11" t="inlineStr">
@@ -14356,12 +14432,16 @@
         <f>IF(F30&gt;0, G30/F30, IF(G30&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J30" s="33" t="inlineStr"/>
+      <c r="J30" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K30" s="34" t="n">
         <v>1280</v>
       </c>
       <c r="L30" s="35" t="n">
-        <v>1280</v>
+        <v>1920</v>
       </c>
       <c r="M30" s="34" t="n">
         <v>1920</v>
@@ -14387,7 +14467,11 @@
         <f>R30-Q30</f>
         <v/>
       </c>
-      <c r="T30" s="37" t="inlineStr"/>
+      <c r="T30" s="37" t="inlineStr">
+        <is>
+          <t>Se habían adelantodo algunos litros a agosto.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="11" t="inlineStr">
@@ -14424,7 +14508,7 @@
         <f>IF(F31&gt;0, G31/F31, IF(G31&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J31" s="33" t="inlineStr"/>
+      <c r="J31" s="33" t="n"/>
       <c r="K31" s="34" t="n">
         <v>100</v>
       </c>
@@ -14455,7 +14539,7 @@
         <f>R31-Q31</f>
         <v/>
       </c>
-      <c r="T31" s="37" t="inlineStr"/>
+      <c r="T31" s="37" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="11" t="inlineStr">
@@ -14492,7 +14576,11 @@
         <f>IF(F32&gt;0, G32/F32, IF(G32&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J32" s="33" t="inlineStr"/>
+      <c r="J32" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K32" s="34" t="n">
         <v>0</v>
       </c>
@@ -14523,7 +14611,11 @@
         <f>R32-Q32</f>
         <v/>
       </c>
-      <c r="T32" s="37" t="inlineStr"/>
+      <c r="T32" s="37" t="inlineStr">
+        <is>
+          <t>Retraso en pedidos, pienso que por retraso en siembras, suele ser estable las ventas de este producto.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="11" t="inlineStr">
@@ -14560,7 +14652,7 @@
         <f>IF(F33&gt;0, G33/F33, IF(G33&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J33" s="33" t="inlineStr"/>
+      <c r="J33" s="33" t="n"/>
       <c r="K33" s="34" t="n">
         <v>0</v>
       </c>
@@ -14591,7 +14683,7 @@
         <f>R33-Q33</f>
         <v/>
       </c>
-      <c r="T33" s="37" t="inlineStr"/>
+      <c r="T33" s="37" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="11" t="inlineStr">
@@ -14628,7 +14720,7 @@
         <f>IF(F34&gt;0, G34/F34, IF(G34&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J34" s="33" t="inlineStr"/>
+      <c r="J34" s="33" t="n"/>
       <c r="K34" s="34" t="n">
         <v>100</v>
       </c>
@@ -14659,7 +14751,7 @@
         <f>R34-Q34</f>
         <v/>
       </c>
-      <c r="T34" s="37" t="inlineStr"/>
+      <c r="T34" s="37" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="11" t="inlineStr">
@@ -14696,7 +14788,7 @@
         <f>IF(F35&gt;0, G35/F35, IF(G35&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J35" s="33" t="inlineStr"/>
+      <c r="J35" s="33" t="n"/>
       <c r="K35" s="34" t="n">
         <v>0</v>
       </c>
@@ -14727,7 +14819,7 @@
         <f>R35-Q35</f>
         <v/>
       </c>
-      <c r="T35" s="37" t="inlineStr"/>
+      <c r="T35" s="37" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="11" t="inlineStr">
@@ -14764,7 +14856,11 @@
         <f>IF(F36&gt;0, G36/F36, IF(G36&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J36" s="33" t="inlineStr"/>
+      <c r="J36" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K36" s="34" t="n">
         <v>5120</v>
       </c>
@@ -14795,7 +14891,11 @@
         <f>R36-Q36</f>
         <v/>
       </c>
-      <c r="T36" s="37" t="inlineStr"/>
+      <c r="T36" s="37" t="inlineStr">
+        <is>
+          <t>Van con Stock y por temas de Auditorías no han querido realizar pedidos en Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="11" t="inlineStr">
@@ -14832,7 +14932,7 @@
         <f>IF(F37&gt;0, G37/F37, IF(G37&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J37" s="33" t="inlineStr"/>
+      <c r="J37" s="33" t="n"/>
       <c r="K37" s="34" t="n">
         <v>0</v>
       </c>
@@ -14863,7 +14963,11 @@
         <f>R37-Q37</f>
         <v/>
       </c>
-      <c r="T37" s="37" t="inlineStr"/>
+      <c r="T37" s="37" t="inlineStr">
+        <is>
+          <t>Es un cliente en concreto el que se lo lleva, este año no lo ha pedido.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="11" t="inlineStr">
@@ -14900,7 +15004,7 @@
         <f>IF(F38&gt;0, G38/F38, IF(G38&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J38" s="33" t="inlineStr"/>
+      <c r="J38" s="33" t="n"/>
       <c r="K38" s="34" t="n">
         <v>0</v>
       </c>
@@ -14931,7 +15035,7 @@
         <f>R38-Q38</f>
         <v/>
       </c>
-      <c r="T38" s="37" t="inlineStr"/>
+      <c r="T38" s="37" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="11" t="inlineStr">
@@ -14968,7 +15072,7 @@
         <f>IF(F39&gt;0, G39/F39, IF(G39&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J39" s="33" t="inlineStr"/>
+      <c r="J39" s="33" t="n"/>
       <c r="K39" s="34" t="n">
         <v>0</v>
       </c>
@@ -14999,7 +15103,7 @@
         <f>R39-Q39</f>
         <v/>
       </c>
-      <c r="T39" s="37" t="inlineStr"/>
+      <c r="T39" s="37" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="11" t="inlineStr">
@@ -15036,7 +15140,7 @@
         <f>IF(F40&gt;0, G40/F40, IF(G40&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J40" s="33" t="inlineStr"/>
+      <c r="J40" s="33" t="n"/>
       <c r="K40" s="34" t="n">
         <v>0</v>
       </c>
@@ -15067,7 +15171,7 @@
         <f>R40-Q40</f>
         <v/>
       </c>
-      <c r="T40" s="37" t="inlineStr"/>
+      <c r="T40" s="37" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="11" t="inlineStr">
@@ -15104,12 +15208,16 @@
         <f>IF(F41&gt;0, G41/F41, IF(G41&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J41" s="33" t="inlineStr"/>
+      <c r="J41" s="33" t="inlineStr">
+        <is>
+          <t>Adelanto de pedidos</t>
+        </is>
+      </c>
       <c r="K41" s="34" t="n">
         <v>900</v>
       </c>
       <c r="L41" s="35" t="n">
-        <v>900</v>
+        <v>1200</v>
       </c>
       <c r="M41" s="34" t="n">
         <v>0</v>
@@ -15135,7 +15243,11 @@
         <f>R41-Q41</f>
         <v/>
       </c>
-      <c r="T41" s="37" t="inlineStr"/>
+      <c r="T41" s="37" t="inlineStr">
+        <is>
+          <t>Se adelantaron a Agosto los pedidos</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="11" t="inlineStr">
@@ -15172,7 +15284,7 @@
         <f>IF(F42&gt;0, G42/F42, IF(G42&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J42" s="33" t="inlineStr"/>
+      <c r="J42" s="33" t="n"/>
       <c r="K42" s="34" t="n">
         <v>400</v>
       </c>
@@ -15203,7 +15315,7 @@
         <f>R42-Q42</f>
         <v/>
       </c>
-      <c r="T42" s="37" t="inlineStr"/>
+      <c r="T42" s="37" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="11" t="inlineStr">
@@ -15240,7 +15352,7 @@
         <f>IF(F43&gt;0, G43/F43, IF(G43&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J43" s="33" t="inlineStr"/>
+      <c r="J43" s="33" t="n"/>
       <c r="K43" s="34" t="n">
         <v>0</v>
       </c>
@@ -15271,7 +15383,7 @@
         <f>R43-Q43</f>
         <v/>
       </c>
-      <c r="T43" s="37" t="inlineStr"/>
+      <c r="T43" s="37" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="B44" s="11" t="inlineStr">
@@ -15308,12 +15420,16 @@
         <f>IF(F44&gt;0, G44/F44, IF(G44&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J44" s="33" t="inlineStr"/>
+      <c r="J44" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K44" s="34" t="n">
         <v>0</v>
       </c>
       <c r="L44" s="35" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="M44" s="34" t="n">
         <v>0</v>
@@ -15339,7 +15455,7 @@
         <f>R44-Q44</f>
         <v/>
       </c>
-      <c r="T44" s="37" t="inlineStr"/>
+      <c r="T44" s="37" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="B45" s="11" t="inlineStr">
@@ -15376,12 +15492,16 @@
         <f>IF(F45&gt;0, G45/F45, IF(G45&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J45" s="33" t="inlineStr"/>
+      <c r="J45" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K45" s="34" t="n">
         <v>300</v>
       </c>
       <c r="L45" s="35" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="M45" s="34" t="n">
         <v>0</v>
@@ -15407,7 +15527,11 @@
         <f>R45-Q45</f>
         <v/>
       </c>
-      <c r="T45" s="37" t="inlineStr"/>
+      <c r="T45" s="37" t="inlineStr">
+        <is>
+          <t>Van con Stock y por temas de Auditorías no han querido realizar pedidos en Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="B46" s="11" t="inlineStr">
@@ -15444,7 +15568,7 @@
         <f>IF(F46&gt;0, G46/F46, IF(G46&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J46" s="33" t="inlineStr"/>
+      <c r="J46" s="33" t="n"/>
       <c r="K46" s="34" t="n">
         <v>0</v>
       </c>
@@ -15475,7 +15599,7 @@
         <f>R46-Q46</f>
         <v/>
       </c>
-      <c r="T46" s="37" t="inlineStr"/>
+      <c r="T46" s="37" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="B47" s="11" t="inlineStr">
@@ -15512,7 +15636,11 @@
         <f>IF(F47&gt;0, G47/F47, IF(G47&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J47" s="33" t="inlineStr"/>
+      <c r="J47" s="33" t="inlineStr">
+        <is>
+          <t>Adelanto de pedidos</t>
+        </is>
+      </c>
       <c r="K47" s="34" t="n">
         <v>1280</v>
       </c>
@@ -15543,7 +15671,11 @@
         <f>R47-Q47</f>
         <v/>
       </c>
-      <c r="T47" s="37" t="inlineStr"/>
+      <c r="T47" s="37" t="inlineStr">
+        <is>
+          <t>Se habían adelantodo algunos litros a agosto.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="B48" s="11" t="inlineStr">
@@ -15580,18 +15712,22 @@
         <f>IF(F48&gt;0, G48/F48, IF(G48&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J48" s="33" t="inlineStr"/>
+      <c r="J48" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K48" s="34" t="n">
         <v>1280</v>
       </c>
       <c r="L48" s="35" t="n">
-        <v>1280</v>
+        <v>3200</v>
       </c>
       <c r="M48" s="34" t="n">
         <v>1920</v>
       </c>
       <c r="N48" s="35" t="n">
-        <v>1920</v>
+        <v>1280</v>
       </c>
       <c r="O48" s="34" t="n">
         <v>1280</v>
@@ -15611,7 +15747,11 @@
         <f>R48-Q48</f>
         <v/>
       </c>
-      <c r="T48" s="37" t="inlineStr"/>
+      <c r="T48" s="37" t="inlineStr">
+        <is>
+          <t>Por motivos de Auditorías no han querido realizar pedidos en Septiembre</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="B49" s="11" t="inlineStr">
@@ -15648,7 +15788,7 @@
         <f>IF(F49&gt;0, G49/F49, IF(G49&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J49" s="33" t="inlineStr"/>
+      <c r="J49" s="33" t="n"/>
       <c r="K49" s="34" t="n">
         <v>0</v>
       </c>
@@ -15679,7 +15819,7 @@
         <f>R49-Q49</f>
         <v/>
       </c>
-      <c r="T49" s="37" t="inlineStr"/>
+      <c r="T49" s="37" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="B50" s="11" t="inlineStr">
@@ -15716,7 +15856,7 @@
         <f>IF(F50&gt;0, G50/F50, IF(G50&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J50" s="33" t="inlineStr"/>
+      <c r="J50" s="33" t="n"/>
       <c r="K50" s="34" t="n">
         <v>0</v>
       </c>
@@ -15747,7 +15887,7 @@
         <f>R50-Q50</f>
         <v/>
       </c>
-      <c r="T50" s="37" t="inlineStr"/>
+      <c r="T50" s="37" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="B51" s="11" t="inlineStr">
@@ -15784,7 +15924,7 @@
         <f>IF(F51&gt;0, G51/F51, IF(G51&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J51" s="33" t="inlineStr"/>
+      <c r="J51" s="33" t="n"/>
       <c r="K51" s="34" t="n">
         <v>640</v>
       </c>
@@ -15815,7 +15955,7 @@
         <f>R51-Q51</f>
         <v/>
       </c>
-      <c r="T51" s="37" t="inlineStr"/>
+      <c r="T51" s="37" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="B52" s="11" t="inlineStr">
@@ -15852,7 +15992,7 @@
         <f>IF(F52&gt;0, G52/F52, IF(G52&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J52" s="33" t="inlineStr"/>
+      <c r="J52" s="33" t="n"/>
       <c r="K52" s="34" t="n">
         <v>0</v>
       </c>
@@ -15883,7 +16023,7 @@
         <f>R52-Q52</f>
         <v/>
       </c>
-      <c r="T52" s="37" t="inlineStr"/>
+      <c r="T52" s="37" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="B53" s="11" t="inlineStr">
@@ -15920,12 +16060,16 @@
         <f>IF(F53&gt;0, G53/F53, IF(G53&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J53" s="33" t="inlineStr"/>
+      <c r="J53" s="33" t="inlineStr">
+        <is>
+          <t>Atraso de pedidos</t>
+        </is>
+      </c>
       <c r="K53" s="34" t="n">
         <v>0</v>
       </c>
       <c r="L53" s="35" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M53" s="34" t="n">
         <v>100</v>
@@ -15951,7 +16095,7 @@
         <f>R53-Q53</f>
         <v/>
       </c>
-      <c r="T53" s="37" t="inlineStr"/>
+      <c r="T53" s="37" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="B54" s="11" t="inlineStr">
@@ -15988,7 +16132,11 @@
         <f>IF(F54&gt;0, G54/F54, IF(G54&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J54" s="33" t="inlineStr"/>
+      <c r="J54" s="33" t="inlineStr">
+        <is>
+          <t>Otro motivo</t>
+        </is>
+      </c>
       <c r="K54" s="34" t="n">
         <v>2480</v>
       </c>
@@ -16019,7 +16167,11 @@
         <f>R54-Q54</f>
         <v/>
       </c>
-      <c r="T54" s="37" t="inlineStr"/>
+      <c r="T54" s="37" t="inlineStr">
+        <is>
+          <t>Salió una operación de jaulas para un cliente, lo que merma la compra de garrafas de 20l</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="B55" s="11" t="inlineStr">
@@ -16091,7 +16243,7 @@
         <f>R55-Q55</f>
         <v/>
       </c>
-      <c r="T55" s="37" t="inlineStr"/>
+      <c r="T55" s="37" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="B56" s="11" t="inlineStr">
@@ -16128,7 +16280,7 @@
         <f>IF(F56&gt;0, G56/F56, IF(G56&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J56" s="33" t="inlineStr"/>
+      <c r="J56" s="33" t="n"/>
       <c r="K56" s="34" t="n">
         <v>0</v>
       </c>
@@ -16159,7 +16311,7 @@
         <f>R56-Q56</f>
         <v/>
       </c>
-      <c r="T56" s="37" t="inlineStr"/>
+      <c r="T56" s="37" t="n"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="B57" s="11" t="inlineStr">
@@ -16196,7 +16348,7 @@
         <f>IF(F57&gt;0, G57/F57, IF(G57&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J57" s="33" t="inlineStr"/>
+      <c r="J57" s="33" t="n"/>
       <c r="K57" s="34" t="n">
         <v>0</v>
       </c>
@@ -16227,7 +16379,7 @@
         <f>R57-Q57</f>
         <v/>
       </c>
-      <c r="T57" s="37" t="inlineStr"/>
+      <c r="T57" s="37" t="n"/>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="B58" s="11" t="inlineStr">
@@ -16264,7 +16416,7 @@
         <f>IF(F58&gt;0, G58/F58, IF(G58&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J58" s="33" t="inlineStr"/>
+      <c r="J58" s="33" t="n"/>
       <c r="K58" s="34" t="n">
         <v>300</v>
       </c>
@@ -16295,7 +16447,7 @@
         <f>R58-Q58</f>
         <v/>
       </c>
-      <c r="T58" s="37" t="inlineStr"/>
+      <c r="T58" s="37" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="B59" s="11" t="inlineStr">
@@ -16332,7 +16484,7 @@
         <f>IF(F59&gt;0, G59/F59, IF(G59&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J59" s="33" t="inlineStr"/>
+      <c r="J59" s="33" t="n"/>
       <c r="K59" s="34" t="n">
         <v>640</v>
       </c>
@@ -16349,7 +16501,7 @@
         <v>0</v>
       </c>
       <c r="P59" s="35" t="n">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="Q59" s="12">
         <f>K59+M59+O59</f>
@@ -16363,7 +16515,7 @@
         <f>R59-Q59</f>
         <v/>
       </c>
-      <c r="T59" s="37" t="inlineStr"/>
+      <c r="T59" s="37" t="n"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="B60" s="11" t="inlineStr">
@@ -16400,7 +16552,7 @@
         <f>IF(F60&gt;0, G60/F60, IF(G60&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J60" s="33" t="inlineStr"/>
+      <c r="J60" s="33" t="n"/>
       <c r="K60" s="34" t="n">
         <v>0</v>
       </c>
@@ -16431,7 +16583,7 @@
         <f>R60-Q60</f>
         <v/>
       </c>
-      <c r="T60" s="37" t="inlineStr"/>
+      <c r="T60" s="37" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="B61" s="11" t="inlineStr">
@@ -16468,18 +16620,18 @@
         <f>IF(F61&gt;0, G61/F61, IF(G61&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J61" s="33" t="inlineStr"/>
+      <c r="J61" s="33" t="n"/>
       <c r="K61" s="34" t="n">
         <v>0</v>
       </c>
       <c r="L61" s="35" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="M61" s="34" t="n">
         <v>0</v>
       </c>
       <c r="N61" s="35" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="O61" s="34" t="n">
         <v>300</v>
@@ -16499,7 +16651,7 @@
         <f>R61-Q61</f>
         <v/>
       </c>
-      <c r="T61" s="37" t="inlineStr"/>
+      <c r="T61" s="37" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="B62" s="11" t="inlineStr">
@@ -16536,7 +16688,7 @@
         <f>IF(F62&gt;0, G62/F62, IF(G62&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J62" s="33" t="inlineStr"/>
+      <c r="J62" s="33" t="n"/>
       <c r="K62" s="34" t="n">
         <v>108</v>
       </c>
@@ -16567,7 +16719,7 @@
         <f>R62-Q62</f>
         <v/>
       </c>
-      <c r="T62" s="37" t="inlineStr"/>
+      <c r="T62" s="37" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="B63" s="11" t="inlineStr">
@@ -16604,7 +16756,7 @@
         <f>IF(F63&gt;0, G63/F63, IF(G63&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J63" s="33" t="inlineStr"/>
+      <c r="J63" s="33" t="n"/>
       <c r="K63" s="34" t="n">
         <v>0</v>
       </c>
@@ -16635,7 +16787,7 @@
         <f>R63-Q63</f>
         <v/>
       </c>
-      <c r="T63" s="37" t="inlineStr"/>
+      <c r="T63" s="37" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="B64" s="11" t="inlineStr">
@@ -16672,7 +16824,7 @@
         <f>IF(F64&gt;0, G64/F64, IF(G64&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J64" s="33" t="inlineStr"/>
+      <c r="J64" s="33" t="n"/>
       <c r="K64" s="34" t="n">
         <v>100</v>
       </c>
@@ -16703,7 +16855,7 @@
         <f>R64-Q64</f>
         <v/>
       </c>
-      <c r="T64" s="37" t="inlineStr"/>
+      <c r="T64" s="37" t="n"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="B65" s="11" t="inlineStr">
@@ -16740,7 +16892,7 @@
         <f>IF(F65&gt;0, G65/F65, IF(G65&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J65" s="33" t="inlineStr"/>
+      <c r="J65" s="33" t="n"/>
       <c r="K65" s="34" t="n">
         <v>0</v>
       </c>
@@ -16771,7 +16923,7 @@
         <f>R65-Q65</f>
         <v/>
       </c>
-      <c r="T65" s="37" t="inlineStr"/>
+      <c r="T65" s="37" t="n"/>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="B66" s="11" t="inlineStr">
@@ -16808,7 +16960,7 @@
         <f>IF(F66&gt;0, G66/F66, IF(G66&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J66" s="33" t="inlineStr"/>
+      <c r="J66" s="33" t="n"/>
       <c r="K66" s="34" t="n">
         <v>40</v>
       </c>
@@ -16839,7 +16991,7 @@
         <f>R66-Q66</f>
         <v/>
       </c>
-      <c r="T66" s="37" t="inlineStr"/>
+      <c r="T66" s="37" t="n"/>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="B67" s="11" t="inlineStr">
@@ -16876,7 +17028,7 @@
         <f>IF(F67&gt;0, G67/F67, IF(G67&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J67" s="33" t="inlineStr"/>
+      <c r="J67" s="33" t="n"/>
       <c r="K67" s="34" t="n">
         <v>0</v>
       </c>
@@ -16907,7 +17059,7 @@
         <f>R67-Q67</f>
         <v/>
       </c>
-      <c r="T67" s="37" t="inlineStr"/>
+      <c r="T67" s="37" t="n"/>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="B68" s="11" t="inlineStr">
@@ -16944,18 +17096,18 @@
         <f>IF(F68&gt;0, G68/F68, IF(G68&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J68" s="33" t="inlineStr"/>
+      <c r="J68" s="33" t="n"/>
       <c r="K68" s="34" t="n">
         <v>0</v>
       </c>
       <c r="L68" s="35" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M68" s="34" t="n">
         <v>100</v>
       </c>
       <c r="N68" s="35" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O68" s="34" t="n">
         <v>200</v>
@@ -16975,7 +17127,7 @@
         <f>R68-Q68</f>
         <v/>
       </c>
-      <c r="T68" s="37" t="inlineStr"/>
+      <c r="T68" s="37" t="n"/>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="B69" s="11" t="inlineStr">
@@ -17012,7 +17164,7 @@
         <f>IF(F69&gt;0, G69/F69, IF(G69&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J69" s="33" t="inlineStr"/>
+      <c r="J69" s="33" t="n"/>
       <c r="K69" s="34" t="n">
         <v>640</v>
       </c>
@@ -17043,7 +17195,7 @@
         <f>R69-Q69</f>
         <v/>
       </c>
-      <c r="T69" s="37" t="inlineStr"/>
+      <c r="T69" s="37" t="n"/>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="B70" s="11" t="inlineStr">
@@ -17080,7 +17232,7 @@
         <f>IF(F70&gt;0, G70/F70, IF(G70&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J70" s="33" t="inlineStr"/>
+      <c r="J70" s="33" t="n"/>
       <c r="K70" s="34" t="n">
         <v>300</v>
       </c>
@@ -17111,7 +17263,7 @@
         <f>R70-Q70</f>
         <v/>
       </c>
-      <c r="T70" s="37" t="inlineStr"/>
+      <c r="T70" s="37" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="B71" s="11" t="inlineStr">
@@ -17157,7 +17309,7 @@
         <v>2760</v>
       </c>
       <c r="L71" s="35" t="n">
-        <v>2760</v>
+        <v>2560</v>
       </c>
       <c r="M71" s="34" t="n">
         <v>1280</v>
@@ -17183,7 +17335,11 @@
         <f>R71-Q71</f>
         <v/>
       </c>
-      <c r="T71" s="37" t="inlineStr"/>
+      <c r="T71" s="37" t="inlineStr">
+        <is>
+          <t>Cliente que va bajo demanda de campo, complicado preveer</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="B72" s="11" t="inlineStr">
@@ -17220,7 +17376,7 @@
         <f>IF(F72&gt;0, G72/F72, IF(G72&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J72" s="33" t="inlineStr"/>
+      <c r="J72" s="33" t="n"/>
       <c r="K72" s="34" t="n">
         <v>0</v>
       </c>
@@ -17251,7 +17407,7 @@
         <f>R72-Q72</f>
         <v/>
       </c>
-      <c r="T72" s="37" t="inlineStr"/>
+      <c r="T72" s="37" t="n"/>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="B73" s="11" t="inlineStr">
@@ -17323,7 +17479,11 @@
         <f>R73-Q73</f>
         <v/>
       </c>
-      <c r="T73" s="37" t="inlineStr"/>
+      <c r="T73" s="37" t="inlineStr">
+        <is>
+          <t>Cliente que va bajo demanda de campo, complicado preveer</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="25" customHeight="1">
       <c r="B74" s="38" t="inlineStr">

</xml_diff>